<commit_message>
updated homepage test data
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/TestData.xlsx
+++ b/src/test/resources/testdata/TestData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Automation Practice\Automation Framework Design\OrangeHRMProject_V1\src\test\resources\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E69324B-D30A-4925-825F-71E4457BEBCF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{46D0F3F0-1062-40C8-91C9-46EA2995DAC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="10">
   <si>
     <t>Username</t>
   </si>
@@ -388,7 +388,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B3"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.26953125" bestFit="1" customWidth="1"/>
@@ -412,11 +412,35 @@
       </c>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="B3" s="1"/>
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" t="s">
+        <v>2</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>3</v>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B2" r:id="rId1" xr:uid="{1101C664-9A1A-4124-8FD0-BD2C1D31B1E4}"/>
+    <hyperlink ref="B3" r:id="rId2" xr:uid="{378E0A82-BFC7-4055-BA47-017573AB43E1}"/>
+    <hyperlink ref="B4" r:id="rId3" xr:uid="{9FD965B7-51BA-4A1D-8997-D38B004D444B}"/>
+    <hyperlink ref="B5" r:id="rId4" xr:uid="{62F9E591-7F31-4BBF-B931-844CCA6D1535}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>